<commit_message>
Reassess MICAS unmet need against actual retrieval log
Reconcile P37 demand with the actual MICAS activity data. Key findings:
MICAS delivers ~405 ICU-level retrievals/yr (86% from ICU, 51% on
vasopressors), East ~67%; 11.6% decline rate, ~54% of declines supply-side
(capacity/hours). Service is 99% in-hours, ~4.3h per job. First-pass
'enhanced need' proxy (~5,500/yr) re-anchored to a high-acuity denominator;
defensible unmet-need range ~400-1,100 critical-care transfers/yr.

Adds aggregate workbook tabs 10-12 and a reassessment section. Raw MICAS
file is NOT committed (contains consultant names + patient DOB/age).

https://claude.ai/code/session_015ktyuND4oS6cFwwbehgWn4
</commit_message>
<xml_diff>
--- a/analysis/MICAS_unmet_need_analysis.xlsx
+++ b/analysis/MICAS_unmet_need_analysis.xlsx
@@ -17,6 +17,9 @@
     <sheet name="7_OutOfPerformance" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="8_Coverage_Unmet_MODEL" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="9_DoW_x_Hour" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="10_MICAS_actual" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="11_Declines_categorised" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="12_Reconciliation" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1125,6 +1128,354 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>MICAS actual (aggregate)</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Delivered retrievals (12mo, Jun25-May26)</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Referrals (12mo)</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Declined (12mo)</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Decline rate %</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>11.6</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Delivered by team - East</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Delivered by team - West</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Delivered by team - South</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Referrals in-hours 08:00-19:59 %</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Mean team commitment per retrieval (h)</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>4.3</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Referred from ICU %</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>On vasopressors %</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Sedated/paralysed (ventilated) %</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Arterial line %</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>83</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Decline reason (categorised, names removed)</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>No team available (capacity)</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Out-of-hours / would overrun</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>No reason recorded</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Clinically not MICAS-appropriate (correct gatekeeping)</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Cohort</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Annualised</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>MICAS delivered (actual)</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>~410-470</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>ICU-to-ICU ventilated/pressor retrieval</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>MICAS declined - capacity/hours (measured floor)</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>~30-55</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>~54% of declines are supply-side, not clinical</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>P37 37D03 "inappropriate for NAS" (narrowest high-acuity)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>~800</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>NAS itself flags as beyond P37 remit</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>P37 Delta + special equipment (broad ICU proxy)</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>~3,700</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>AMPDS proxy; overstates true ICU-level</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>P37 adult + any enhanced need (first-pass, too broad)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>~5,500</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Superseded by MICAS-data reality</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -2516,7 +2867,6 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr"/>
       <c r="B5" t="n">
         <v>513</v>
       </c>

</xml_diff>

<commit_message>
Add out-of-hours / extra-team recovery model
Discrete-event simulation of MICAS-appropriate demand across rota options,
using actual MICAS job durations (~4.3h) and calibrated to the actual ~405
retrievals/yr baseline (demand ~900/yr central, 700-1100 sensitivity):

  C1 weekend teams      +35/yr
  C2 evenings to 24:00  +161/yr  (best value)
  C3 full 24/7          +291/yr
  C4 24/7 + 4th team    +303/yr

Priority ladder: evenings -> full 24/7 -> 4th team for peak resilience.
Adds workbook tab 13 and recovery scenarios chart.
</commit_message>
<xml_diff>
--- a/analysis/MICAS_unmet_need_analysis.xlsx
+++ b/analysis/MICAS_unmet_need_analysis.xlsx
@@ -20,6 +20,7 @@
     <sheet name="10_MICAS_actual" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="11_Declines_categorised" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="12_Reconciliation" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="13_Recovery_scenarios" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1476,6 +1477,142 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Rota configuration</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Served/yr @ D=700</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Served/yr @ D=900</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Served/yr @ D=1100</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Recovered/yr (central)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>C0  Current (3 wkdy/1 wkend, 08–20)</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>405</v>
+      </c>
+      <c r="C2" t="n">
+        <v>405</v>
+      </c>
+      <c r="D2" t="n">
+        <v>405</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>C1  +Weekend teams (3 teams 7d, 08–20)</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>429</v>
+      </c>
+      <c r="C3" t="n">
+        <v>440</v>
+      </c>
+      <c r="D3" t="n">
+        <v>445</v>
+      </c>
+      <c r="E3" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>C2  +Evenings (3 teams 7d, 08–24)</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>549</v>
+      </c>
+      <c r="C4" t="n">
+        <v>566</v>
+      </c>
+      <c r="D4" t="n">
+        <v>574</v>
+      </c>
+      <c r="E4" t="n">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>C3  24/7 (3 teams round-clock)</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>676</v>
+      </c>
+      <c r="C5" t="n">
+        <v>696</v>
+      </c>
+      <c r="D5" t="n">
+        <v>709</v>
+      </c>
+      <c r="E5" t="n">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>C4  24/7 + 4th team</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>684</v>
+      </c>
+      <c r="C6" t="n">
+        <v>708</v>
+      </c>
+      <c r="D6" t="n">
+        <v>728</v>
+      </c>
+      <c r="E6" t="n">
+        <v>303</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Model East two-tier expansion permutations
East-focused discrete-event model with two tiers (MICAS Acute co-located
vs hospital-composite), confirmed by bimodal mobilisation in the data
(52% <=25min vs 32% >=45min). Cork & Galway held constant (regional, no
expansion). Recovery vs current ~270/yr:

  P1 Acute every weekday        +~24
  P2 +2nd team 08-20            +~79
  P3 +2nd team 10-22            +~110  (~9 evening)
  P4 +2nd team 12-00            +~130  (~24 evening)
  P5 +2nd team 12-00 Acute 5d   +~155  (~37 evening)

Second East team on a 12:00-00:00 shift recovers most and uniquely covers
the evening 20:00-24:00 peak (uncovered today). Adds workbook tab 14 and
two figures.
</commit_message>
<xml_diff>
--- a/analysis/MICAS_unmet_need_analysis.xlsx
+++ b/analysis/MICAS_unmet_need_analysis.xlsx
@@ -21,6 +21,7 @@
     <sheet name="11_Declines_categorised" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="12_Reconciliation" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="13_Recovery_scenarios" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="14_East_permutations" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1613,6 +1614,142 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A6:E11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Recovered_per_yr_central</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Range_low</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Range_high</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>of_which_evening_2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>P1  Acute every weekday (1 team, 08–20)</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>24</v>
+      </c>
+      <c r="C7" t="n">
+        <v>19</v>
+      </c>
+      <c r="D7" t="n">
+        <v>28</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>P2  + 2nd team 08–20</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>79</v>
+      </c>
+      <c r="C8" t="n">
+        <v>60</v>
+      </c>
+      <c r="D8" t="n">
+        <v>100</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>P3  + 2nd team 10–22</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>111</v>
+      </c>
+      <c r="C9" t="n">
+        <v>76</v>
+      </c>
+      <c r="D9" t="n">
+        <v>141</v>
+      </c>
+      <c r="E9" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>P4  + 2nd team 12–00</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>132</v>
+      </c>
+      <c r="C10" t="n">
+        <v>92</v>
+      </c>
+      <c r="D10" t="n">
+        <v>166</v>
+      </c>
+      <c r="E10" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>P5  + 2nd team 12–00, Acute all 5 days</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>156</v>
+      </c>
+      <c r="C11" t="n">
+        <v>120</v>
+      </c>
+      <c r="D11" t="n">
+        <v>180</v>
+      </c>
+      <c r="E11" t="n">
+        <v>37</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add historical MICAS analysis (1996-2025): supply saturation
Analyse four historical workbooks (2024 national + East/South/West 2025
logs). Key findings:
- National activity plateaued ~346-360/yr for 2022-2025 after COVID peak
  of 469 (2021); growth decade 104->469. Flat output + ~23% decline rate
  = supply-capped, not demand-capped.
- 2024: 360 delivered, 107 declined (~23%). Team split East 214 (59%),
  West 83 (23%), South 63 (18%, -25% YoY).
- Staff-restrictions log: repeated whole-day 'no service' from single
  absences (South 'no consultant', West 'nurse ill') -> small-team
  fragility; supports no S/W expansion + East resilience.
- Validates model params: 100% ventilated; job medians East 3.3h/South
  4.4h/West 5.6h; mobilisation bimodal (East)/fast(South)/slow(West).
Adds workbook tabs 15-16 and two trend charts. Raw files not committed
(retain DOB/age/gender).
</commit_message>
<xml_diff>
--- a/analysis/MICAS_unmet_need_analysis.xlsx
+++ b/analysis/MICAS_unmet_need_analysis.xlsx
@@ -22,6 +22,8 @@
     <sheet name="12_Reconciliation" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="13_Recovery_scenarios" sheetId="14" state="visible" r:id="rId14"/>
     <sheet name="14_East_permutations" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="15_Historical_trend" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="16_Team_split_decline" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1750,6 +1752,366 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Transfers</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1996</v>
+      </c>
+      <c r="B2" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1997</v>
+      </c>
+      <c r="B3" t="n">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1998</v>
+      </c>
+      <c r="B4" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>1999</v>
+      </c>
+      <c r="B5" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2000</v>
+      </c>
+      <c r="B6" t="n">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>2001</v>
+      </c>
+      <c r="B7" t="n">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>2002</v>
+      </c>
+      <c r="B8" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>2003</v>
+      </c>
+      <c r="B9" t="n">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>2004</v>
+      </c>
+      <c r="B10" t="n">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>2005</v>
+      </c>
+      <c r="B11" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>2006</v>
+      </c>
+      <c r="B12" t="n">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>2007</v>
+      </c>
+      <c r="B13" t="n">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>2008</v>
+      </c>
+      <c r="B14" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>2009</v>
+      </c>
+      <c r="B15" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>2010</v>
+      </c>
+      <c r="B16" t="n">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>2011</v>
+      </c>
+      <c r="B17" t="n">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>2012</v>
+      </c>
+      <c r="B18" t="n">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>2013</v>
+      </c>
+      <c r="B19" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>2014</v>
+      </c>
+      <c r="B20" t="n">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>2015</v>
+      </c>
+      <c r="B21" t="n">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>2016</v>
+      </c>
+      <c r="B22" t="n">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>2017</v>
+      </c>
+      <c r="B23" t="n">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>2018</v>
+      </c>
+      <c r="B24" t="n">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>2019</v>
+      </c>
+      <c r="B25" t="n">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>2020</v>
+      </c>
+      <c r="B26" t="n">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B27" t="n">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>2022</v>
+      </c>
+      <c r="B28" t="n">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B29" t="n">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B30" t="n">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B31" t="n">
+        <v>356</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A8:C13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2024 outcome</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Transferred (delivered)</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>360</v>
+      </c>
+      <c r="C9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Declined</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>107</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>~23% of referrals</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Deferred</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>~10</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Stood down</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>~9</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Not transferred</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>2</v>
+      </c>
+      <c r="C13" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Decode hospital codes; add corridor + distance analysis
Apply hospital crosswalk (code->name + geocodes) to MICAS data:
- Decode corridors: Mayo->Galway (66km), Beaumont->Mater (5km),
  Galway<->Beaumont (189km), Kerry->CUH (91km); Dublin dominant hub.
- Distance by team: East median 41km, South 84km, West 118km.
- Distance drives job length (r=0.61): 0-50km=3.3h ... 150km+=6.4h.
- Quantifies the overrun mechanism: explains Cork/Galway long-distance
  declines, West's lower throughput, and why a 2nd East team (short hops,
  ~3.3h) is the most throughput-efficient expansion.
- 2 UK/out-of-state transfers identified.
Adds workbook tab 17 and corridor flow map.
</commit_message>
<xml_diff>
--- a/analysis/MICAS_unmet_need_analysis.xlsx
+++ b/analysis/MICAS_unmet_need_analysis.xlsx
@@ -24,6 +24,7 @@
     <sheet name="14_East_permutations" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="15_Historical_trend" sheetId="16" state="visible" r:id="rId16"/>
     <sheet name="16_Team_split_decline" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="17_Corridors_decoded" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2053,7 +2054,6 @@
       <c r="B9" t="n">
         <v>360</v>
       </c>
-      <c r="C9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2081,7 +2081,6 @@
           <t>~10</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2094,7 +2093,6 @@
           <t>~9</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2105,7 +2103,762 @@
       <c r="B13" t="n">
         <v>2</v>
       </c>
-      <c r="C13" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D41"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>From</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>To</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Dist_km</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Mayo University Hospital</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>University Hospital Galway</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>20</v>
+      </c>
+      <c r="D2" t="n">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Beaumont Hospital</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Mater Misericordiae University Hospital</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>15</v>
+      </c>
+      <c r="D3" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Naas General Hospital</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Tallaght University Hospital</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>11</v>
+      </c>
+      <c r="D4" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Beaumont Hospital</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>St James’ Hospital</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>10</v>
+      </c>
+      <c r="D5" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Bandon Community Hospital</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Cork University Hospital</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>9</v>
+      </c>
+      <c r="D6" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Midland Regional Hospital Portlaoise</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>St James’ Hospital</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>9</v>
+      </c>
+      <c r="D7" t="n">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>University Hospital Galway</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Beaumont Hospital</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>9</v>
+      </c>
+      <c r="D8" t="n">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Beaumont Hospital</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Tallaght University Hospital</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>8</v>
+      </c>
+      <c r="D9" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Our Lady of Lourdes Hospital, Drogheda</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Mater Misericordiae University Hospital</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>8</v>
+      </c>
+      <c r="D10" t="n">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>University Hospital Galway</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Mayo University Hospital</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>8</v>
+      </c>
+      <c r="D11" t="n">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Beaumont Hospital</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>University Hospital Galway</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>7</v>
+      </c>
+      <c r="D12" t="n">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Beaumont Hospital</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Our Lady of Lourdes Hospital, Drogheda</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>7</v>
+      </c>
+      <c r="D13" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Cork University Hospital</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>University Hospital Limerick</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>6</v>
+      </c>
+      <c r="D14" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Midland Regional Hospital Mullingar</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Mater Misericordiae University Hospital</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>6</v>
+      </c>
+      <c r="D15" t="n">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>University Hospital Kerry</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Cork University Hospital</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>6</v>
+      </c>
+      <c r="D16" t="n">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>St Vincent’s University Hospital</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Beaumont Hospital</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>6</v>
+      </c>
+      <c r="D17" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>University Hospital Galway</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Sligo University Hospital</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>6</v>
+      </c>
+      <c r="D18" t="n">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Connolly Hospital Blanchardstown</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Mater Misericordiae University Hospital</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>5</v>
+      </c>
+      <c r="D19" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>St Vincent’s University Hospital</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Mater Misericordiae University Hospital</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>5</v>
+      </c>
+      <c r="D20" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Portiuncula University Hospital</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>University Hospital Galway</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>5</v>
+      </c>
+      <c r="D21" t="n">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Beaumont Hospital</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>St Vincent’s University Hospital</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>5</v>
+      </c>
+      <c r="D22" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Our Lady of Lourdes Hospital, Drogheda</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Beaumont Hospital</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>5</v>
+      </c>
+      <c r="D23" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Tallaght University Hospital</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Mater Misericordiae University Hospital</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>5</v>
+      </c>
+      <c r="D24" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Sligo University Hospital</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Mater Misericordiae University Hospital</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>5</v>
+      </c>
+      <c r="D25" t="n">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Beaumont Hospital</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Connolly Hospital Blanchardstown</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>4</v>
+      </c>
+      <c r="D26" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Midland Regional Hospital Mullingar</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>St James’ Hospital</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>4</v>
+      </c>
+      <c r="D27" t="n">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>St Luke’s General Hospital Carlow Kilkenny</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Mater Misericordiae University Hospital</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>4</v>
+      </c>
+      <c r="D28" t="n">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>St Luke’s General Hospital Carlow Kilkenny</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>University Hospital Waterford</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>4</v>
+      </c>
+      <c r="D29" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Connolly Hospital Blanchardstown</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>St James’ Hospital</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>4</v>
+      </c>
+      <c r="D30" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Tallaght University Hospital</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>St James’ Hospital</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>4</v>
+      </c>
+      <c r="D31" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Cork University Hospital</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Mater Misericordiae University Hospital</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>4</v>
+      </c>
+      <c r="D32" t="n">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Beaumont Hospital</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>St Luke’s General Hospital Carlow Kilkenny</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>4</v>
+      </c>
+      <c r="D33" t="n">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Mater Misericordiae University Hospital</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Beaumont Hospital</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>4</v>
+      </c>
+      <c r="D34" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Midland Regional Hospital Portlaoise</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Tallaght University Hospital</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>3</v>
+      </c>
+      <c r="D35" t="n">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Wexford General Hospital</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Mater Misericordiae University Hospital</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>3</v>
+      </c>
+      <c r="D36" t="n">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>University Hospital Limerick</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>University Hospital Galway</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>3</v>
+      </c>
+      <c r="D37" t="n">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>University Hospital Limerick</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Mater Misericordiae University Hospital</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>3</v>
+      </c>
+      <c r="D38" t="n">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>University Hospital Waterford</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>St Vincent’s University Hospital</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>3</v>
+      </c>
+      <c r="D39" t="n">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>St James’ Hospital</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>St Luke’s General Hospital Carlow Kilkenny</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>3</v>
+      </c>
+      <c r="D40" t="n">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Tallaght University Hospital</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Midland Regional Hospital Tullamore</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>3</v>
+      </c>
+      <c r="D41" t="n">
+        <v>74</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>